<commit_message>
Framework-first revision: placeholder KPI numbers, private delivery scoreboard, punctuation scrub
All number KPIs become placeholders pending bottom-up agreement with Ivan.
Delivery Scoreboard moves out of the shared tracker into its own file
(tracker stays team-visible, scores stay private). Em dashes and middot
separators removed from all copy.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RGX7fKtxmHSTi6NvK3idJW
</commit_message>
<xml_diff>
--- a/team-performance/Executive_Project_Tracker_v2.xlsx
+++ b/team-performance/Executive_Project_Tracker_v2.xlsx
@@ -10,14 +10,13 @@
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Master Rollup" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Delivery Scoreboard" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="KPI Targets H2" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="JV" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Anton" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Manzil" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="Elias" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="Jastin" sheetId="9" state="visible" r:id="rId11"/>
-    <sheet name="KPI Key Drivers" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="KPI Targets H2" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="JV" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Anton" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Manzil" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Elias" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Jastin" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="KPI Key Drivers" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -29,12 +28,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="785" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="766" uniqueCount="306">
   <si>
     <t xml:space="preserve">Executive Project Tracker v2, POS Product Team (H2 2026)</t>
   </si>
   <si>
-    <t xml:space="preserve">One file. One tab per owner plus a consolidated Master. Linked to the PBT Metric Tree KPIs agreed with Ivan.</t>
+    <t xml:space="preserve">One file, shared with the whole team. One tab per owner plus a consolidated Master. Linked to the PBT Metric Tree KPIs discussed with Ivan.</t>
   </si>
   <si>
     <t xml:space="preserve">Purpose</t>
@@ -46,19 +45,22 @@
     <t xml:space="preserve">This sheet is the executive-level view: what the project is, whether it is moving, what it is expected to move (Impact), and whether we delivered when we said we would.</t>
   </si>
   <si>
+    <t xml:space="preserve">Everyone sees everything here. The point is a single, centralized view of what the team is doing.</t>
+  </si>
+  <si>
     <t xml:space="preserve">What is new in v2 (after the 29 Jun KPI alignment with Ivan)</t>
   </si>
   <si>
-    <t xml:space="preserve">Impact (bottom-up): every project carries the estimated business impact and its assumption, e.g. "salvage ~20% of rejects -&gt; +P6M/mo Deals disb". Targets come from agreed actions, never out of nowhere.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Due and Delivered: the date agreed with the owner, and the date it actually shipped. This is the delivery track record Ivan asked for - delivery is managed by business result, not by number of emails sent.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delivery Scoreboard tab: per-owner on-time rate, computed automatically. This is each owner's D3 delivery KPI and the evidence base for the quarterly scorecard (Speed).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KPI Targets H2 tab: the per-line volume and PBT targets, target vs actual by month. Yellow cells are to be agreed on the Ivan call or filled monthly from Nhat's PBT model and Jenny's dashboard.</t>
+    <t xml:space="preserve">Impact (bottom-up): every project carries the estimated business impact and its assumption. Targets come from agreed actions, never out of nowhere.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Due and Delivered: the date agreed with the owner, and the date it actually shipped. Delivery is managed by business result, not by number of emails sent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KPI Targets H2 tab: per-line targets, target vs actual by month. All number targets are placeholders for now; yellow cells are set bottom-up and agreed with Ivan, then filled monthly.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delivery track record: Due and Delivered feed a separate Delivery Scoreboard file kept by Kurt. The shared work is visible to all; individual delivery scores stay private.</t>
   </si>
   <si>
     <t xml:space="preserve">The tabs</t>
@@ -67,10 +69,7 @@
     <t xml:space="preserve">Master Rollup: every project across all owners, ranked. Keep this Viewer-only for the team.</t>
   </si>
   <si>
-    <t xml:space="preserve">KPI Targets H2: line-level targets (Tier 0/1) - review monthly.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delivery Scoreboard: delivery track record per owner - review weekly at standup.</t>
+    <t xml:space="preserve">KPI Targets H2: line-level targets (Tier 0 and Tier 1), reviewed monthly.</t>
   </si>
   <si>
     <t xml:space="preserve">One tab per owner (JV, Anton, Manzil, Elias, Jastin). Each person maintains only their own tab.</t>
@@ -112,13 +111,13 @@
     <t xml:space="preserve">Operating cadence</t>
   </si>
   <si>
-    <t xml:space="preserve">Weekly standup: walk the Master top-down - blocked and overdue first - and update Due/Delivered. Details live in ClickUp via the link column.</t>
+    <t xml:space="preserve">Weekly standup: walk the Master top-down, blocked and overdue first, and update Due and Delivered. Details live in ClickUp via the link column.</t>
   </si>
   <si>
     <t xml:space="preserve">Monthly: KPI readout on the KPI Targets H2 tab against Nhat's PBT-per-line model and Jenny's metric-tree dashboard.</t>
   </si>
   <si>
-    <t xml:space="preserve">Quarterly: individual reviews on the QuantumLight (Revolut) Product Owner scorecard - Culture, Skills, and Deliverables = (Speed + Quality) x Complexity. The Delivery Scoreboard and Impact column are the evidence for Speed and business impact. A-players calibrated to 15-25% of the team.</t>
+    <t xml:space="preserve">Quarterly: individual reviews on the QuantumLight (Revolut) Product Owner scorecard. Culture, Skills, and Deliverables = (Speed + Quality) x Complexity. The Impact column and the private Delivery Scoreboard are the evidence for business impact and Speed. A-players calibrated to 15-25% of the team.</t>
   </si>
   <si>
     <t xml:space="preserve">Lock each tab to one person (done inside Google Sheets)</t>
@@ -220,7 +219,7 @@
     <t xml:space="preserve">Credit Line - D1 Utilization &amp; drawdown</t>
   </si>
   <si>
-    <t xml:space="preserve">CL utilization &amp; drawdown - target set ~15 Aug (30d post-launch)</t>
+    <t xml:space="preserve">CL utilization and drawdown, target set ~30 days post-launch</t>
   </si>
   <si>
     <t xml:space="preserve">Launched 15 Jul (F&amp;F/ETB). Phase-1 open: repayment/statement emails, eligibility, biz events, web FAQ, pending-txn spec. Refund/chargeback &amp; IPP later phases.</t>
@@ -238,7 +237,7 @@
     <t xml:space="preserve">Motorcycles - D1 Moto monthly disbursement</t>
   </si>
   <si>
-    <t xml:space="preserve">Moto ~P15M/mo run rate (gated by Nhat)</t>
+    <t xml:space="preserve">Moto monthly run rate, gated by Nhat</t>
   </si>
   <si>
     <t xml:space="preserve">Addendum &amp; SA guide done, delivered via SAP. refresher pending. return-config changes being finalized.</t>
@@ -253,7 +252,7 @@
     <t xml:space="preserve">Deals - D1 Monthly disbursement</t>
   </si>
   <si>
-    <t xml:space="preserve">Conversion lift on low-risk base - size w/ Nhat before comms</t>
+    <t xml:space="preserve">Conversion lift on low-risk base, size with Nhat before comms</t>
   </si>
   <si>
     <t xml:space="preserve">Additional-limit offer to low-risk clients to lift conversion. DE deployed. comms Jul 20.</t>
@@ -298,7 +297,7 @@
     <t xml:space="preserve">Deals BD - D2 New merchants live &amp; disbursing</t>
   </si>
   <si>
-    <t xml:space="preserve">New merchants live &amp; disbursing; ticket uplift P1,000-2,000</t>
+    <t xml:space="preserve">New merchants live and disbursing, ticket uplift</t>
   </si>
   <si>
     <t xml:space="preserve">Brand pipeline. WARM: Kimstore, 3Cat, Hati, Laptop Factory, Samsung, PrimerGrp, PowerMac, AirAsia, Qoala. Rejected: MetroMart, Engkanto, DataBlitz, Vivo, Mandaue Foam.</t>
@@ -313,7 +312,7 @@
     <t xml:space="preserve">Card - D2 Card unit economics</t>
   </si>
   <si>
-    <t xml:space="preserve">Per-card break-even on interchange @ CAC P300-500</t>
+    <t xml:space="preserve">Per-card break-even on interchange at target CAC</t>
   </si>
   <si>
     <t xml:space="preserve">BillEase Mastercard (numberless) w/ AUB &amp; MatchMove. MOA negotiation (audit cap, CS cert, VAPT). design + bureau RFPs out. activation BRD done. Target prod Q4 2026.</t>
@@ -364,7 +363,7 @@
     <t xml:space="preserve">QRPh - D1 Monthly disbursement run rate</t>
   </si>
   <si>
-    <t xml:space="preserve">Protects QRPh ~P107M/mo run rate</t>
+    <t xml:space="preserve">Protects the QRPh run rate</t>
   </si>
   <si>
     <t xml:space="preserve">Daily QRPh chargeback escalation &amp; checking for AUB and Netbank.</t>
@@ -514,7 +513,7 @@
     <t xml:space="preserve">Integrate Merchant Guide to Billease Docs</t>
   </si>
   <si>
-    <t xml:space="preserve">~30% fewer onboarding tickets</t>
+    <t xml:space="preserve">Fewer onboarding tickets via self-serve guide</t>
   </si>
   <si>
     <t xml:space="preserve">Single self-service Merchant Guide: handbook + 7 walkthroughs, vector screens, PII redaction. Target 30% fewer tickets.</t>
@@ -610,198 +609,162 @@
     <t xml:space="preserve">https://app.clickup.com/t/9008174123/86ey2gvyt</t>
   </si>
   <si>
-    <t xml:space="preserve">Delivery Scoreboard, per owner (D3 delivery KPI)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ivan, 29 Jun: manage delivery by the track record of agreed steps shipped on pace, and by business impact, not activity. Computed from each owner tab (Due / Delivered / Status).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Committed (Due set)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">On time</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Late</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Overdue (open)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">On-time rate</t>
+    <t xml:space="preserve">KPI Targets H2 2026, per line (Tier 0 / Tier 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Framework first: every target cell is a placeholder until agreed with Ivan. Bottom-up: current state -&gt; diagnosis -&gt; agreed actions -&gt; estimated impact -&gt; timeline. Yellow = set on the Ivan call or fill monthly (volumes: Jenny's dashboard; PBT: Nhat's model).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line outcomes, monthly volume (PHP M disbursement)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nov</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YTD att.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basis / notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QRPh disbursement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Star</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jastin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run-rate target to confirm with Ivan. Hold and defend the star line (chargebacks, onboarding cycle time).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   actual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deals disbursement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Question</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anton + Manzil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Staged monthly ramp at positive NPM. Stage sizes and timing to agree; the reject-salvage plan sizes the ramp.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moto (KServico)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run-rate target gated by Nhat's unit-economics check.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deals, managed accounts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manzil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ProTech, Maxicare, 3Cat. Ticket uplift target to agree.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Credit Line (utilization %, target set ~30 days post-launch)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CL utilization / drawdown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New launch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Launched 15 Jul (F&amp;F/ETB). Baseline first, then set the target with Ivan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tier 0, PBT per line (PHP M, from Nhat's model)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QRPh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w/ Nhat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From Nhat's model once live.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Online</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maintain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moto / Deals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phase says push volume, watch NPM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Credit Line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model rows live post-launch.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kill or keep decision pending.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Offline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash cow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maintain, no PM by design.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Milestones (dates, not monthly numbers)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Milestone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done</t>
   </si>
   <si>
     <t xml:space="preserve">Notes</t>
   </si>
   <si>
-    <t xml:space="preserve">Team</t>
-  </si>
-  <si>
-    <t xml:space="preserve">How to read it: Committed = rows with an agreed Due date. On-time rate = on time / (on time + late). Overdue (open) = past Due, not shipped, not cancelled.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Due is set when the step is agreed with the owner (standup or ClickUp), Delivered when it ships. Backfill both every Monday. Most rows are yellow today - first pass is due at the 21 Jul standup.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feeds the quarterly Revolut-style scorecard: Speed &lt;- on-time rate; Quality &lt;- iterations to done (ClickUp reopens); Complexity &lt;- precedent, judged per project. Deliverables = (Speed + Quality) x Complexity.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KPI Targets H2 2026, per line (Tier 0 / Tier 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bottom-up targets: current state -&gt; diagnosis -&gt; agreed actions -&gt; estimated impact -&gt; timeline. Yellow = agree on the Ivan call, or fill monthly (volumes: Jenny's dashboard; PBT: Nhat's model).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Line outcomes, monthly volume (P M disbursement)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Line</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aug</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nov</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dec</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YTD att.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Basis / notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QRPh disbursement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Star</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jastin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Run-rate ~P107M/mo per KPI tab; hold and defend (chargebacks, onboarding cycle time).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   actual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deals disbursement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Question</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anton + Manzil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Staged P25M -&gt; 50M -&gt; 100M/mo at positive NPM; agree stage timing with Ivan. Salvage plan on rejects sizes the ramp.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Moto (KServico)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~P15M/mo, gated by Nhat's unit-economics check.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deals, managed accounts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manzil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ProTech, Maxicare, 3Cat; ticket uplift P1,000-2,000.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Credit Line (utilization %, set ~15 Aug, 30d post-launch)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CL utilization / drawdown</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New launch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elias</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Launched 15 Jul (F&amp;F/ETB). Baseline first, then set target with Ivan ~15 Aug.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tier 0, PBT per line (P M, from Nhat's model)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QRPh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w/ Nhat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">May-26 read: small positive.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Online</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maintain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">May-26 read: possibly positive, small.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Moto / Deals</t>
-  </si>
-  <si>
-    <t xml:space="preserve">May-26 read: calculated negative; long-run unknown. Phase says push volume, watch NPM.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Credit Line</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Model rows live post-launch.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kill-or-keep decision pending.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Offline</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cash cow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maintain; no PM assigned by design.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Milestones (dates, not monthly numbers)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Milestone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Done</t>
-  </si>
-  <si>
     <t xml:space="preserve">Solar: kill-or-keep decision</t>
   </si>
   <si>
@@ -823,7 +786,7 @@
     <t xml:space="preserve">Card launch</t>
   </si>
   <si>
-    <t xml:space="preserve">Target Sep per KPI tab; prod Q4 per Access Card row.</t>
+    <t xml:space="preserve">Target Sep per KPI tab, prod Q4 2026 per Access Card row.</t>
   </si>
   <si>
     <t xml:space="preserve">PBT-per-line model live, monthly</t>
@@ -844,25 +807,25 @@
     <t xml:space="preserve">One source for this tab.</t>
   </si>
   <si>
-    <t xml:space="preserve">JV: edit only this tab. Yellow = fill me (Impact &amp; Due before In Progress; Delivered when shipped).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anton: edit only this tab. Yellow = fill me (Impact &amp; Due before In Progress; Delivered when shipped).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manzil: edit only this tab. Yellow = fill me (Impact &amp; Due before In Progress; Delivered when shipped).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elias: edit only this tab. Yellow = fill me (Impact &amp; Due before In Progress; Delivered when shipped).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jastin: edit only this tab. Yellow = fill me (Impact &amp; Due before In Progress; Delivered when shipped).</t>
+    <t xml:space="preserve">JV: edit only this tab. Yellow = fill me (Impact and Due before In Progress; Delivered when shipped).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anton: edit only this tab. Yellow = fill me (Impact and Due before In Progress; Delivered when shipped).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manzil: edit only this tab. Yellow = fill me (Impact and Due before In Progress; Delivered when shipped).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elias: edit only this tab. Yellow = fill me (Impact and Due before In Progress; Delivered when shipped).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jastin: edit only this tab. Yellow = fill me (Impact and Due before In Progress; Delivered when shipped).</t>
   </si>
   <si>
     <t xml:space="preserve">KPI Key Drivers, PBT Metric Tree (H2 2026)</t>
   </si>
   <si>
-    <t xml:space="preserve">Each owner carries 3 metrics: line outcome, key driver, delivery. The KPI column on each tab points here.</t>
+    <t xml:space="preserve">Each owner carries 3 metrics: line outcome, key driver, delivery. Number targets are placeholders (TBD) until agreed with Ivan; they live on KPI Targets H2.</t>
   </si>
   <si>
     <t xml:space="preserve">Line(s)</t>
@@ -880,7 +843,7 @@
     <t xml:space="preserve">Deals and Solar (product)</t>
   </si>
   <si>
-    <t xml:space="preserve">Deals monthly disbursement at positive NPM (staged 25M, 50M, 100M)</t>
+    <t xml:space="preserve">Deals monthly disbursement at positive NPM (staged ramp, stage targets TBD)</t>
   </si>
   <si>
     <t xml:space="preserve">Deals acceptance and conversion rate (salvage plan on rejects)</t>
@@ -895,7 +858,7 @@
     <t xml:space="preserve">Deals disbursement from managed accounts (ProTech, Maxicare, 3Cat)</t>
   </si>
   <si>
-    <t xml:space="preserve">New merchants live and disbursing. Ticket uplift to PHP 1,000 to 2,000</t>
+    <t xml:space="preserve">New merchants live and disbursing. Ticket uplift target TBD</t>
   </si>
   <si>
     <t xml:space="preserve">Delivery on BD pipeline commitments</t>
@@ -904,10 +867,10 @@
     <t xml:space="preserve">Motorcycles and Sales Agent Portal</t>
   </si>
   <si>
-    <t xml:space="preserve">Moto (KServico) monthly disbursement (about 15M per month, gated by Nhat)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Disbursement per active sales agent (PHP 315K to 500K plus)</t>
+    <t xml:space="preserve">Moto (KServico) monthly disbursement (run-rate target TBD, gated by Nhat)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disbursement per active sales agent (uplift target TBD)</t>
   </si>
   <si>
     <t xml:space="preserve">Delivery on SAP milestones, voucher and quiz modules</t>
@@ -919,7 +882,7 @@
     <t xml:space="preserve">Credit line utilization and drawdown (set 30 days post-launch)</t>
   </si>
   <si>
-    <t xml:space="preserve">Card unit economics: per-card break-even on interchange at CAC PHP 300 to 500</t>
+    <t xml:space="preserve">Card unit economics: per-card break-even on interchange (CAC target TBD)</t>
   </si>
   <si>
     <t xml:space="preserve">Delivery on launch milestones (CL 15 Jul, card Sep)</t>
@@ -928,7 +891,7 @@
     <t xml:space="preserve">QRPh and Merchant Onboarding</t>
   </si>
   <si>
-    <t xml:space="preserve">QRPh monthly disbursement run rate (about 107M per month, star line)</t>
+    <t xml:space="preserve">QRPh monthly disbursement run rate (target TBD, star line)</t>
   </si>
   <si>
     <t xml:space="preserve">Onboarding cycle time (signed to live), zero config errors</t>
@@ -982,21 +945,20 @@
     <t xml:space="preserve">Delivery incl. recurring-defect elimination (iOS QR, selfie KYC)</t>
   </si>
   <si>
-    <t xml:space="preserve">Targets and monthly actuals live on the KPI Targets H2 tab. Delivery (D3) is scored on the Delivery Scoreboard tab.</t>
+    <t xml:space="preserve">Targets and monthly actuals live on the KPI Targets H2 tab. Delivery (D3) is scored by Kurt in the separate Delivery Scoreboard file.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd\ mmm"/>
-    <numFmt numFmtId="166" formatCode="General"/>
+    <numFmt numFmtId="166" formatCode="#,##0"/>
     <numFmt numFmtId="167" formatCode="0%"/>
-    <numFmt numFmtId="168" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1085,13 +1047,6 @@
       <b val="true"/>
       <sz val="10"/>
       <color rgb="FF1E8E5A"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1196,7 +1151,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1277,23 +1232,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1309,15 +1252,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1325,7 +1260,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1333,7 +1268,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1633,13 +1568,13 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="3" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1658,13 +1593,13 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="3" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1786,198 +1721,6 @@
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="2" t="s">
         <v>35</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:E14"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="40"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="35" t="s">
-        <v>37</v>
-      </c>
-      <c r="B4" s="35" t="s">
-        <v>278</v>
-      </c>
-      <c r="C4" s="35" t="s">
-        <v>279</v>
-      </c>
-      <c r="D4" s="35" t="s">
-        <v>280</v>
-      </c>
-      <c r="E4" s="35" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="36" t="s">
-        <v>54</v>
-      </c>
-      <c r="B5" s="37" t="s">
-        <v>282</v>
-      </c>
-      <c r="C5" s="37" t="s">
-        <v>283</v>
-      </c>
-      <c r="D5" s="37" t="s">
-        <v>284</v>
-      </c>
-      <c r="E5" s="37" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="36" t="s">
-        <v>86</v>
-      </c>
-      <c r="B6" s="37" t="s">
-        <v>286</v>
-      </c>
-      <c r="C6" s="37" t="s">
-        <v>287</v>
-      </c>
-      <c r="D6" s="37" t="s">
-        <v>288</v>
-      </c>
-      <c r="E6" s="37" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="36" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" s="37" t="s">
-        <v>290</v>
-      </c>
-      <c r="C7" s="37" t="s">
-        <v>291</v>
-      </c>
-      <c r="D7" s="37" t="s">
-        <v>292</v>
-      </c>
-      <c r="E7" s="37" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="36" t="s">
-        <v>60</v>
-      </c>
-      <c r="B8" s="37" t="s">
-        <v>294</v>
-      </c>
-      <c r="C8" s="37" t="s">
-        <v>295</v>
-      </c>
-      <c r="D8" s="37" t="s">
-        <v>296</v>
-      </c>
-      <c r="E8" s="37" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="36" t="s">
-        <v>101</v>
-      </c>
-      <c r="B9" s="37" t="s">
-        <v>298</v>
-      </c>
-      <c r="C9" s="37" t="s">
-        <v>299</v>
-      </c>
-      <c r="D9" s="37" t="s">
-        <v>300</v>
-      </c>
-      <c r="E9" s="37" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="36" t="s">
-        <v>302</v>
-      </c>
-      <c r="B10" s="37" t="s">
-        <v>303</v>
-      </c>
-      <c r="C10" s="37" t="s">
-        <v>304</v>
-      </c>
-      <c r="D10" s="37" t="s">
-        <v>305</v>
-      </c>
-      <c r="E10" s="37" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="36" t="s">
-        <v>307</v>
-      </c>
-      <c r="B11" s="37" t="s">
-        <v>308</v>
-      </c>
-      <c r="C11" s="37" t="s">
-        <v>309</v>
-      </c>
-      <c r="D11" s="37" t="s">
-        <v>310</v>
-      </c>
-      <c r="E11" s="37" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="36" t="s">
-        <v>312</v>
-      </c>
-      <c r="B12" s="37" t="s">
-        <v>313</v>
-      </c>
-      <c r="C12" s="37" t="s">
-        <v>314</v>
-      </c>
-      <c r="D12" s="37" t="s">
-        <v>315</v>
-      </c>
-      <c r="E12" s="37" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
-        <v>317</v>
       </c>
     </row>
   </sheetData>
@@ -3096,259 +2839,6 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="64"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="B5" s="20" t="n">
-        <f aca="false">COUNT(JV!F4:F400)</f>
-        <v>0</v>
-      </c>
-      <c r="C5" s="20" t="n">
-        <f aca="false">COUNT(JV!G4:G400)</f>
-        <v>2</v>
-      </c>
-      <c r="D5" s="20" t="n">
-        <f aca="false">SUMPRODUCT((JV!G4:G400&lt;&gt;"")*(JV!F4:F400&lt;&gt;"")*(JV!G4:G400&lt;=JV!F4:F400))</f>
-        <v>0</v>
-      </c>
-      <c r="E5" s="20" t="n">
-        <f aca="false">SUMPRODUCT((JV!G4:G400&lt;&gt;"")*(JV!F4:F400&lt;&gt;"")*(JV!G4:G400&gt;JV!F4:F400))</f>
-        <v>0</v>
-      </c>
-      <c r="F5" s="20" t="n">
-        <f aca="true">SUMPRODUCT((JV!F4:F400&lt;&gt;"")*(JV!G4:G400="")*(JV!B4:B400&lt;&gt;"Completed")*(JV!B4:B400&lt;&gt;"Cancelled")*(JV!F4:F400&lt;TODAY()))</f>
-        <v>0</v>
-      </c>
-      <c r="G5" s="21" t="str">
-        <f aca="false">IF(D5+E5=0,"-",D5/(D5+E5))</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
-        <v>54</v>
-      </c>
-      <c r="B6" s="20" t="n">
-        <f aca="false">COUNT(Anton!F4:F400)</f>
-        <v>1</v>
-      </c>
-      <c r="C6" s="20" t="n">
-        <f aca="false">COUNT(Anton!G4:G400)</f>
-        <v>0</v>
-      </c>
-      <c r="D6" s="20" t="n">
-        <f aca="false">SUMPRODUCT((Anton!G4:G400&lt;&gt;"")*(Anton!F4:F400&lt;&gt;"")*(Anton!G4:G400&lt;=Anton!F4:F400))</f>
-        <v>0</v>
-      </c>
-      <c r="E6" s="20" t="n">
-        <f aca="false">SUMPRODUCT((Anton!G4:G400&lt;&gt;"")*(Anton!F4:F400&lt;&gt;"")*(Anton!G4:G400&gt;Anton!F4:F400))</f>
-        <v>0</v>
-      </c>
-      <c r="F6" s="20" t="n">
-        <f aca="true">SUMPRODUCT((Anton!F4:F400&lt;&gt;"")*(Anton!G4:G400="")*(Anton!B4:B400&lt;&gt;"Completed")*(Anton!B4:B400&lt;&gt;"Cancelled")*(Anton!F4:F400&lt;TODAY()))</f>
-        <v>0</v>
-      </c>
-      <c r="G6" s="21" t="str">
-        <f aca="false">IF(D6+E6=0,"-",D6/(D6+E6))</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="B7" s="20" t="n">
-        <f aca="false">COUNT(Manzil!F4:F400)</f>
-        <v>0</v>
-      </c>
-      <c r="C7" s="20" t="n">
-        <f aca="false">COUNT(Manzil!G4:G400)</f>
-        <v>1</v>
-      </c>
-      <c r="D7" s="20" t="n">
-        <f aca="false">SUMPRODUCT((Manzil!G4:G400&lt;&gt;"")*(Manzil!F4:F400&lt;&gt;"")*(Manzil!G4:G400&lt;=Manzil!F4:F400))</f>
-        <v>0</v>
-      </c>
-      <c r="E7" s="20" t="n">
-        <f aca="false">SUMPRODUCT((Manzil!G4:G400&lt;&gt;"")*(Manzil!F4:F400&lt;&gt;"")*(Manzil!G4:G400&gt;Manzil!F4:F400))</f>
-        <v>0</v>
-      </c>
-      <c r="F7" s="20" t="n">
-        <f aca="true">SUMPRODUCT((Manzil!F4:F400&lt;&gt;"")*(Manzil!G4:G400="")*(Manzil!B4:B400&lt;&gt;"Completed")*(Manzil!B4:B400&lt;&gt;"Cancelled")*(Manzil!F4:F400&lt;TODAY()))</f>
-        <v>0</v>
-      </c>
-      <c r="G7" s="21" t="str">
-        <f aca="false">IF(D7+E7=0,"-",D7/(D7+E7))</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
-        <v>60</v>
-      </c>
-      <c r="B8" s="20" t="n">
-        <f aca="false">COUNT(Elias!F4:F400)</f>
-        <v>0</v>
-      </c>
-      <c r="C8" s="20" t="n">
-        <f aca="false">COUNT(Elias!G4:G400)</f>
-        <v>0</v>
-      </c>
-      <c r="D8" s="20" t="n">
-        <f aca="false">SUMPRODUCT((Elias!G4:G400&lt;&gt;"")*(Elias!F4:F400&lt;&gt;"")*(Elias!G4:G400&lt;=Elias!F4:F400))</f>
-        <v>0</v>
-      </c>
-      <c r="E8" s="20" t="n">
-        <f aca="false">SUMPRODUCT((Elias!G4:G400&lt;&gt;"")*(Elias!F4:F400&lt;&gt;"")*(Elias!G4:G400&gt;Elias!F4:F400))</f>
-        <v>0</v>
-      </c>
-      <c r="F8" s="20" t="n">
-        <f aca="true">SUMPRODUCT((Elias!F4:F400&lt;&gt;"")*(Elias!G4:G400="")*(Elias!B4:B400&lt;&gt;"Completed")*(Elias!B4:B400&lt;&gt;"Cancelled")*(Elias!F4:F400&lt;TODAY()))</f>
-        <v>0</v>
-      </c>
-      <c r="G8" s="21" t="str">
-        <f aca="false">IF(D8+E8=0,"-",D8/(D8+E8))</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="B9" s="20" t="n">
-        <f aca="false">COUNT(Jastin!F4:F400)</f>
-        <v>0</v>
-      </c>
-      <c r="C9" s="20" t="n">
-        <f aca="false">COUNT(Jastin!G4:G400)</f>
-        <v>0</v>
-      </c>
-      <c r="D9" s="20" t="n">
-        <f aca="false">SUMPRODUCT((Jastin!G4:G400&lt;&gt;"")*(Jastin!F4:F400&lt;&gt;"")*(Jastin!G4:G400&lt;=Jastin!F4:F400))</f>
-        <v>0</v>
-      </c>
-      <c r="E9" s="20" t="n">
-        <f aca="false">SUMPRODUCT((Jastin!G4:G400&lt;&gt;"")*(Jastin!F4:F400&lt;&gt;"")*(Jastin!G4:G400&gt;Jastin!F4:F400))</f>
-        <v>0</v>
-      </c>
-      <c r="F9" s="20" t="n">
-        <f aca="true">SUMPRODUCT((Jastin!F4:F400&lt;&gt;"")*(Jastin!G4:G400="")*(Jastin!B4:B400&lt;&gt;"Completed")*(Jastin!B4:B400&lt;&gt;"Cancelled")*(Jastin!F4:F400&lt;TODAY()))</f>
-        <v>0</v>
-      </c>
-      <c r="G9" s="21" t="str">
-        <f aca="false">IF(D9+E9=0,"-",D9/(D9+E9))</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="B10" s="22" t="n">
-        <f aca="false">SUM(B5:B9)</f>
-        <v>1</v>
-      </c>
-      <c r="C10" s="22" t="n">
-        <f aca="false">SUM(C5:C9)</f>
-        <v>3</v>
-      </c>
-      <c r="D10" s="22" t="n">
-        <f aca="false">SUM(D5:D9)</f>
-        <v>0</v>
-      </c>
-      <c r="E10" s="22" t="n">
-        <f aca="false">SUM(E5:E9)</f>
-        <v>0</v>
-      </c>
-      <c r="F10" s="22" t="n">
-        <f aca="false">SUM(F5:F9)</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="23" t="str">
-        <f aca="false">IF(D10+E10=0,"-",D10/(D10+E10))</f>
-        <v>-</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
-        <v>204</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
   <dimension ref="A1:K41"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -3362,595 +2852,571 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>37</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>218</v>
+        <v>206</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>219</v>
+        <v>207</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>220</v>
-      </c>
-      <c r="D6" s="24" t="n">
-        <v>107</v>
-      </c>
-      <c r="E6" s="24" t="n">
-        <v>107</v>
-      </c>
-      <c r="F6" s="24" t="n">
-        <v>107</v>
-      </c>
-      <c r="G6" s="24" t="n">
-        <v>107</v>
-      </c>
-      <c r="H6" s="24" t="n">
-        <v>107</v>
-      </c>
-      <c r="I6" s="24" t="n">
-        <v>107</v>
-      </c>
-      <c r="J6" s="25"/>
-      <c r="K6" s="26" t="s">
-        <v>221</v>
+        <v>208</v>
+      </c>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="23" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="B7" s="25"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28"/>
-      <c r="H7" s="28"/>
-      <c r="I7" s="28"/>
-      <c r="J7" s="29" t="str">
+      <c r="A7" s="24" t="s">
+        <v>210</v>
+      </c>
+      <c r="B7" s="22"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="21"/>
+      <c r="I7" s="21"/>
+      <c r="J7" s="25" t="str">
         <f aca="false">IFERROR(IF(COUNT(D7:I7)=0,"-",SUM(D7:I7)/SUMPRODUCT((D7:I7&lt;&gt;"")*D6:I6)),"-")</f>
         <v>-</v>
       </c>
-      <c r="K7" s="25"/>
+      <c r="K7" s="22"/>
     </row>
     <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>225</v>
-      </c>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="25"/>
-      <c r="K8" s="26" t="s">
-        <v>226</v>
+        <v>213</v>
+      </c>
+      <c r="D8" s="21"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="21"/>
+      <c r="I8" s="21"/>
+      <c r="J8" s="22"/>
+      <c r="K8" s="23" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="B9" s="25"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="28"/>
-      <c r="J9" s="29" t="str">
+      <c r="A9" s="24" t="s">
+        <v>210</v>
+      </c>
+      <c r="B9" s="22"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="21"/>
+      <c r="I9" s="21"/>
+      <c r="J9" s="25" t="str">
         <f aca="false">IFERROR(IF(COUNT(D9:I9)=0,"-",SUM(D9:I9)/SUMPRODUCT((D9:I9&lt;&gt;"")*D8:I8)),"-")</f>
         <v>-</v>
       </c>
-      <c r="K9" s="25"/>
+      <c r="K9" s="22"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>228</v>
-      </c>
-      <c r="D10" s="24" t="n">
-        <v>15</v>
-      </c>
-      <c r="E10" s="24" t="n">
-        <v>15</v>
-      </c>
-      <c r="F10" s="24" t="n">
-        <v>15</v>
-      </c>
-      <c r="G10" s="24" t="n">
-        <v>15</v>
-      </c>
-      <c r="H10" s="24" t="n">
-        <v>15</v>
-      </c>
-      <c r="I10" s="24" t="n">
-        <v>15</v>
-      </c>
-      <c r="J10" s="25"/>
-      <c r="K10" s="26" t="s">
-        <v>229</v>
+        <v>216</v>
+      </c>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="21"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="23" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="B11" s="25"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="28"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="28"/>
-      <c r="I11" s="28"/>
-      <c r="J11" s="29" t="str">
+      <c r="A11" s="24" t="s">
+        <v>210</v>
+      </c>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="21"/>
+      <c r="I11" s="21"/>
+      <c r="J11" s="25" t="str">
         <f aca="false">IFERROR(IF(COUNT(D11:I11)=0,"-",SUM(D11:I11)/SUMPRODUCT((D11:I11&lt;&gt;"")*D10:I10)),"-")</f>
         <v>-</v>
       </c>
-      <c r="K11" s="25"/>
+      <c r="K11" s="22"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>231</v>
-      </c>
-      <c r="D12" s="30"/>
-      <c r="E12" s="30"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="30"/>
-      <c r="I12" s="30"/>
-      <c r="J12" s="25"/>
-      <c r="K12" s="26" t="s">
-        <v>232</v>
+        <v>219</v>
+      </c>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="21"/>
+      <c r="I12" s="21"/>
+      <c r="J12" s="22"/>
+      <c r="K12" s="23" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="B13" s="25"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="28"/>
-      <c r="G13" s="28"/>
-      <c r="H13" s="28"/>
-      <c r="I13" s="28"/>
-      <c r="J13" s="29" t="str">
+      <c r="A13" s="24" t="s">
+        <v>210</v>
+      </c>
+      <c r="B13" s="22"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="21"/>
+      <c r="I13" s="21"/>
+      <c r="J13" s="25" t="str">
         <f aca="false">IFERROR(IF(COUNT(D13:I13)=0,"-",SUM(D13:I13)/SUMPRODUCT((D13:I13&lt;&gt;"")*D12:I12)),"-")</f>
         <v>-</v>
       </c>
-      <c r="K13" s="25"/>
+      <c r="K13" s="22"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>37</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>236</v>
-      </c>
-      <c r="D17" s="31"/>
-      <c r="E17" s="31"/>
-      <c r="F17" s="31"/>
-      <c r="G17" s="31"/>
-      <c r="H17" s="31"/>
-      <c r="I17" s="31"/>
-      <c r="J17" s="25"/>
-      <c r="K17" s="26" t="s">
-        <v>237</v>
+        <v>224</v>
+      </c>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26"/>
+      <c r="I17" s="26"/>
+      <c r="J17" s="22"/>
+      <c r="K17" s="23" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="B18" s="25"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="31"/>
-      <c r="F18" s="31"/>
-      <c r="G18" s="31"/>
-      <c r="H18" s="31"/>
-      <c r="I18" s="31"/>
-      <c r="J18" s="29" t="str">
+      <c r="A18" s="24" t="s">
+        <v>210</v>
+      </c>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="26"/>
+      <c r="I18" s="26"/>
+      <c r="J18" s="25" t="str">
         <f aca="false">IFERROR(IF(COUNT(D18:I18)=0,"-",SUM(D18:I18)/SUMPRODUCT((D18:I18&lt;&gt;"")*D17:I17)),"-")</f>
         <v>-</v>
       </c>
-      <c r="K18" s="25"/>
+      <c r="K18" s="22"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>238</v>
+        <v>226</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>37</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="B22" s="20" t="s">
-        <v>219</v>
+        <v>207</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>240</v>
-      </c>
-      <c r="D22" s="28"/>
-      <c r="E22" s="28"/>
-      <c r="F22" s="28"/>
-      <c r="G22" s="28"/>
-      <c r="H22" s="28"/>
-      <c r="I22" s="28"/>
-      <c r="J22" s="25"/>
-      <c r="K22" s="26" t="s">
-        <v>241</v>
+        <v>228</v>
+      </c>
+      <c r="D22" s="21"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="21"/>
+      <c r="H22" s="21"/>
+      <c r="I22" s="21"/>
+      <c r="J22" s="22"/>
+      <c r="K22" s="23" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="B23" s="25"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="28"/>
-      <c r="H23" s="28"/>
-      <c r="I23" s="28"/>
-      <c r="J23" s="29" t="str">
+      <c r="A23" s="24" t="s">
+        <v>210</v>
+      </c>
+      <c r="B23" s="22"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="21"/>
+      <c r="H23" s="21"/>
+      <c r="I23" s="21"/>
+      <c r="J23" s="25" t="str">
         <f aca="false">IFERROR(IF(COUNT(D23:I23)=0,"-",SUM(D23:I23)/SUMPRODUCT((D23:I23&lt;&gt;"")*D22:I22)),"-")</f>
         <v>-</v>
       </c>
-      <c r="K23" s="25"/>
+      <c r="K23" s="22"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="19" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>243</v>
+        <v>231</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>240</v>
-      </c>
-      <c r="D24" s="28"/>
-      <c r="E24" s="28"/>
-      <c r="F24" s="28"/>
-      <c r="G24" s="28"/>
-      <c r="H24" s="28"/>
-      <c r="I24" s="28"/>
-      <c r="J24" s="25"/>
-      <c r="K24" s="26" t="s">
-        <v>244</v>
+        <v>228</v>
+      </c>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="21"/>
+      <c r="H24" s="21"/>
+      <c r="I24" s="21"/>
+      <c r="J24" s="22"/>
+      <c r="K24" s="23" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="B25" s="25"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="28"/>
-      <c r="E25" s="28"/>
-      <c r="F25" s="28"/>
-      <c r="G25" s="28"/>
-      <c r="H25" s="28"/>
-      <c r="I25" s="28"/>
-      <c r="J25" s="29" t="str">
+      <c r="A25" s="24" t="s">
+        <v>210</v>
+      </c>
+      <c r="B25" s="22"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="21"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="21"/>
+      <c r="J25" s="25" t="str">
         <f aca="false">IFERROR(IF(COUNT(D25:I25)=0,"-",SUM(D25:I25)/SUMPRODUCT((D25:I25&lt;&gt;"")*D24:I24)),"-")</f>
         <v>-</v>
       </c>
-      <c r="K25" s="25"/>
-    </row>
-    <row r="26" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K25" s="22"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="s">
-        <v>245</v>
+        <v>232</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="C26" s="20" t="s">
-        <v>240</v>
-      </c>
-      <c r="D26" s="28"/>
-      <c r="E26" s="28"/>
-      <c r="F26" s="28"/>
-      <c r="G26" s="28"/>
-      <c r="H26" s="28"/>
-      <c r="I26" s="28"/>
-      <c r="J26" s="25"/>
-      <c r="K26" s="26" t="s">
-        <v>246</v>
+        <v>228</v>
+      </c>
+      <c r="D26" s="21"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="21"/>
+      <c r="H26" s="21"/>
+      <c r="I26" s="21"/>
+      <c r="J26" s="22"/>
+      <c r="K26" s="23" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="B27" s="25"/>
-      <c r="C27" s="25"/>
-      <c r="D27" s="28"/>
-      <c r="E27" s="28"/>
-      <c r="F27" s="28"/>
-      <c r="G27" s="28"/>
-      <c r="H27" s="28"/>
-      <c r="I27" s="28"/>
-      <c r="J27" s="29" t="str">
+      <c r="A27" s="24" t="s">
+        <v>210</v>
+      </c>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="21"/>
+      <c r="H27" s="21"/>
+      <c r="I27" s="21"/>
+      <c r="J27" s="25" t="str">
         <f aca="false">IFERROR(IF(COUNT(D27:I27)=0,"-",SUM(D27:I27)/SUMPRODUCT((D27:I27&lt;&gt;"")*D26:I26)),"-")</f>
         <v>-</v>
       </c>
-      <c r="K27" s="25"/>
+      <c r="K27" s="22"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>247</v>
+        <v>234</v>
       </c>
       <c r="B28" s="20" t="s">
+        <v>223</v>
+      </c>
+      <c r="C28" s="20" t="s">
+        <v>228</v>
+      </c>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="21"/>
+      <c r="I28" s="21"/>
+      <c r="J28" s="22"/>
+      <c r="K28" s="23" t="s">
         <v>235</v>
       </c>
-      <c r="C28" s="20" t="s">
-        <v>240</v>
-      </c>
-      <c r="D28" s="28"/>
-      <c r="E28" s="28"/>
-      <c r="F28" s="28"/>
-      <c r="G28" s="28"/>
-      <c r="H28" s="28"/>
-      <c r="I28" s="28"/>
-      <c r="J28" s="25"/>
-      <c r="K28" s="26" t="s">
-        <v>248</v>
-      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="B29" s="25"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="28"/>
-      <c r="I29" s="28"/>
-      <c r="J29" s="29" t="str">
+      <c r="A29" s="24" t="s">
+        <v>210</v>
+      </c>
+      <c r="B29" s="22"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="21"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="21"/>
+      <c r="G29" s="21"/>
+      <c r="H29" s="21"/>
+      <c r="I29" s="21"/>
+      <c r="J29" s="25" t="str">
         <f aca="false">IFERROR(IF(COUNT(D29:I29)=0,"-",SUM(D29:I29)/SUMPRODUCT((D29:I29&lt;&gt;"")*D28:I28)),"-")</f>
         <v>-</v>
       </c>
-      <c r="K29" s="25"/>
+      <c r="K29" s="22"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>249</v>
+        <v>236</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="C30" s="20" t="s">
-        <v>240</v>
-      </c>
-      <c r="D30" s="28"/>
-      <c r="E30" s="28"/>
-      <c r="F30" s="28"/>
-      <c r="G30" s="28"/>
-      <c r="H30" s="28"/>
-      <c r="I30" s="28"/>
-      <c r="J30" s="25"/>
-      <c r="K30" s="26" t="s">
-        <v>250</v>
+        <v>228</v>
+      </c>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
+      <c r="I30" s="21"/>
+      <c r="J30" s="22"/>
+      <c r="K30" s="23" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="B31" s="25"/>
-      <c r="C31" s="25"/>
-      <c r="D31" s="28"/>
-      <c r="E31" s="28"/>
-      <c r="F31" s="28"/>
-      <c r="G31" s="28"/>
-      <c r="H31" s="28"/>
-      <c r="I31" s="28"/>
-      <c r="J31" s="29" t="str">
+      <c r="A31" s="24" t="s">
+        <v>210</v>
+      </c>
+      <c r="B31" s="22"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="21"/>
+      <c r="G31" s="21"/>
+      <c r="H31" s="21"/>
+      <c r="I31" s="21"/>
+      <c r="J31" s="25" t="str">
         <f aca="false">IFERROR(IF(COUNT(D31:I31)=0,"-",SUM(D31:I31)/SUMPRODUCT((D31:I31&lt;&gt;"")*D30:I30)),"-")</f>
         <v>-</v>
       </c>
-      <c r="K31" s="25"/>
+      <c r="K31" s="22"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="19" t="s">
-        <v>251</v>
+        <v>238</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>252</v>
+        <v>239</v>
       </c>
       <c r="C32" s="20" t="s">
+        <v>228</v>
+      </c>
+      <c r="D32" s="21"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="21"/>
+      <c r="G32" s="21"/>
+      <c r="H32" s="21"/>
+      <c r="I32" s="21"/>
+      <c r="J32" s="22"/>
+      <c r="K32" s="23" t="s">
         <v>240</v>
       </c>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="25"/>
-      <c r="K32" s="26" t="s">
-        <v>253</v>
-      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="B33" s="25"/>
-      <c r="C33" s="25"/>
-      <c r="D33" s="28"/>
-      <c r="E33" s="28"/>
-      <c r="F33" s="28"/>
-      <c r="G33" s="28"/>
-      <c r="H33" s="28"/>
-      <c r="I33" s="28"/>
-      <c r="J33" s="29" t="str">
+      <c r="A33" s="24" t="s">
+        <v>210</v>
+      </c>
+      <c r="B33" s="22"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="21"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="21"/>
+      <c r="G33" s="21"/>
+      <c r="H33" s="21"/>
+      <c r="I33" s="21"/>
+      <c r="J33" s="25" t="str">
         <f aca="false">IFERROR(IF(COUNT(D33:I33)=0,"-",SUM(D33:I33)/SUMPRODUCT((D33:I33&lt;&gt;"")*D32:I32)),"-")</f>
         <v>-</v>
       </c>
-      <c r="K33" s="25"/>
+      <c r="K33" s="22"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>254</v>
+        <v>241</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>37</v>
@@ -3959,10 +3425,10 @@
         <v>43</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>200</v>
+        <v>244</v>
       </c>
       <c r="F36" s="5"/>
       <c r="G36" s="5"/>
@@ -3973,69 +3439,69 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="19" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>258</v>
-      </c>
-      <c r="C37" s="32"/>
-      <c r="D37" s="33"/>
-      <c r="E37" s="27" t="s">
-        <v>259</v>
+        <v>246</v>
+      </c>
+      <c r="C37" s="27"/>
+      <c r="D37" s="28"/>
+      <c r="E37" s="24" t="s">
+        <v>247</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="19" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>261</v>
-      </c>
-      <c r="C38" s="34" t="n">
+        <v>249</v>
+      </c>
+      <c r="C38" s="29" t="n">
         <v>46249</v>
       </c>
-      <c r="D38" s="33"/>
-      <c r="E38" s="27" t="s">
-        <v>262</v>
+      <c r="D38" s="28"/>
+      <c r="E38" s="24" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="19" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>236</v>
-      </c>
-      <c r="C39" s="32"/>
-      <c r="D39" s="33"/>
-      <c r="E39" s="27" t="s">
-        <v>264</v>
+        <v>224</v>
+      </c>
+      <c r="C39" s="27"/>
+      <c r="D39" s="28"/>
+      <c r="E39" s="24" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="19" t="s">
-        <v>265</v>
+        <v>253</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>266</v>
-      </c>
-      <c r="C40" s="32"/>
-      <c r="D40" s="33"/>
-      <c r="E40" s="27" t="s">
-        <v>267</v>
+        <v>254</v>
+      </c>
+      <c r="C40" s="27"/>
+      <c r="D40" s="28"/>
+      <c r="E40" s="24" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="19" t="s">
-        <v>268</v>
+        <v>256</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>269</v>
-      </c>
-      <c r="C41" s="32"/>
-      <c r="D41" s="33"/>
-      <c r="E41" s="27" t="s">
-        <v>270</v>
+        <v>257</v>
+      </c>
+      <c r="C41" s="27"/>
+      <c r="D41" s="28"/>
+      <c r="E41" s="24" t="s">
+        <v>258</v>
       </c>
     </row>
   </sheetData>
@@ -4049,7 +3515,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -4070,7 +3536,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>271</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4353,6 +3819,402 @@
       </c>
       <c r="I14" s="7" t="s">
         <v>183</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B4:B400" type="list">
+      <formula1>"Not Started,In Progress,Blocked,Completed,Cancelled"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C4:C400" type="list">
+      <formula1>"Urgent,High,Normal,Low"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:I17"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="46"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="E4" s="9"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="F5" s="15" t="n">
+        <v>46223</v>
+      </c>
+      <c r="G5" s="15"/>
+      <c r="H5" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="I5" s="13" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E6" s="9"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E7" s="9"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="E8" s="9"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="I8" s="7"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="E9" s="9"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="I9" s="13"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E10" s="9"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E11" s="9"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="I11" s="13" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12" s="9"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E13" s="9"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="I13" s="13" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E14" s="9"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="E15" s="9"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="I15" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E16" s="7"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E17" s="13"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="I17" s="13" t="s">
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -4381,7 +4243,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
@@ -4397,7 +4259,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4431,325 +4293,72 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>56</v>
+        <v>87</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>49</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="E4" s="9"/>
+        <v>88</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>89</v>
+      </c>
       <c r="F4" s="10"/>
       <c r="G4" s="11"/>
       <c r="H4" s="7" t="s">
-        <v>58</v>
+        <v>90</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>59</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>72</v>
+        <v>157</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>49</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>67</v>
+        <v>122</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="F5" s="15" t="n">
-        <v>46223</v>
-      </c>
+        <v>158</v>
+      </c>
+      <c r="E5" s="9"/>
+      <c r="F5" s="10"/>
       <c r="G5" s="15"/>
       <c r="H5" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="I5" s="13" t="s">
-        <v>76</v>
-      </c>
+        <v>159</v>
+      </c>
+      <c r="I5" s="13"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>49</v>
+        <v>184</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>174</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E6" s="9"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="11"/>
+        <v>158</v>
+      </c>
+      <c r="E6" s="7"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11" t="n">
+        <v>46213</v>
+      </c>
       <c r="H6" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="E7" s="9"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="I7" s="13" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="E8" s="9"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="I8" s="7"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>136</v>
-      </c>
-      <c r="E9" s="9"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="13" t="s">
-        <v>137</v>
-      </c>
-      <c r="I9" s="13"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E10" s="9"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="I10" s="7" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="E11" s="9"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="I11" s="13" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E12" s="9"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="I12" s="7" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="B13" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="E13" s="9"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="I13" s="13" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="B14" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E14" s="9"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="I14" s="7" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="s">
-        <v>154</v>
-      </c>
-      <c r="B15" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="E15" s="9"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="I15" s="13" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="B16" s="18" t="s">
-        <v>187</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E16" s="7"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="7" t="s">
-        <v>188</v>
-      </c>
-      <c r="I16" s="7" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
-        <v>190</v>
-      </c>
-      <c r="B17" s="18" t="s">
-        <v>187</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="E17" s="13"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="I17" s="13" t="s">
-        <v>192</v>
-      </c>
+        <v>185</v>
+      </c>
+      <c r="I6" s="7"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -4793,7 +4402,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4827,72 +4436,76 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>87</v>
+        <v>61</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>49</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>88</v>
+        <v>62</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>89</v>
+        <v>63</v>
       </c>
       <c r="F4" s="10"/>
       <c r="G4" s="11"/>
       <c r="H4" s="7" t="s">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>91</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>157</v>
+        <v>92</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>49</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>122</v>
+        <v>67</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="E5" s="9"/>
+        <v>93</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>94</v>
+      </c>
       <c r="F5" s="10"/>
       <c r="G5" s="15"/>
       <c r="H5" s="13" t="s">
-        <v>159</v>
-      </c>
-      <c r="I5" s="13"/>
+        <v>95</v>
+      </c>
+      <c r="I5" s="13" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="B6" s="17" t="s">
-        <v>174</v>
+        <v>97</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>56</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11" t="n">
-        <v>46213</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="E6" s="9"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="11"/>
       <c r="H6" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="I6" s="7"/>
+        <v>99</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>100</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -4920,7 +4533,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
@@ -4936,7 +4549,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4970,32 +4583,30 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>61</v>
+        <v>102</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>49</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>63</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="E4" s="9"/>
       <c r="F4" s="10"/>
       <c r="G4" s="11"/>
       <c r="H4" s="7" t="s">
-        <v>64</v>
+        <v>104</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>65</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>49</v>
@@ -5004,41 +4615,158 @@
         <v>67</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>94</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="E5" s="9"/>
       <c r="F5" s="10"/>
       <c r="G5" s="15"/>
       <c r="H5" s="13" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="I5" s="13" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>56</v>
+        <v>109</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>49</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="E6" s="9"/>
+        <v>110</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>111</v>
+      </c>
       <c r="F6" s="10"/>
       <c r="G6" s="11"/>
       <c r="H6" s="7" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>100</v>
+        <v>113</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="E7" s="9"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="E8" s="9"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="F9" s="10"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="I9" s="13" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="E10" s="9"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="E11" s="9"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="I11" s="13" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -5067,253 +4795,183 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="40"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>266</v>
+      </c>
+      <c r="C4" s="30" t="s">
+        <v>267</v>
+      </c>
+      <c r="D4" s="30" t="s">
+        <v>268</v>
+      </c>
+      <c r="E4" s="30" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="31" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="32" t="s">
+        <v>270</v>
+      </c>
+      <c r="C5" s="32" t="s">
+        <v>271</v>
+      </c>
+      <c r="D5" s="32" t="s">
+        <v>272</v>
+      </c>
+      <c r="E5" s="32" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>274</v>
+      </c>
+      <c r="C6" s="32" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="E4" s="9"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="E5" s="9"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="I5" s="13" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="F6" s="10"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="E7" s="9"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="I7" s="13" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="E8" s="9"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>120</v>
+      <c r="D6" s="32" t="s">
+        <v>276</v>
+      </c>
+      <c r="E6" s="32" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>278</v>
+      </c>
+      <c r="C7" s="32" t="s">
+        <v>279</v>
+      </c>
+      <c r="D7" s="32" t="s">
+        <v>280</v>
+      </c>
+      <c r="E7" s="32" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="31" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" s="32" t="s">
+        <v>282</v>
+      </c>
+      <c r="C8" s="32" t="s">
+        <v>283</v>
+      </c>
+      <c r="D8" s="32" t="s">
+        <v>284</v>
+      </c>
+      <c r="E8" s="32" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
-        <v>160</v>
-      </c>
-      <c r="B9" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>161</v>
-      </c>
-      <c r="F9" s="10"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="I9" s="13" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="B10" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="E10" s="9"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="I10" s="7" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
-        <v>167</v>
-      </c>
-      <c r="B11" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="E11" s="9"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="13" t="s">
-        <v>168</v>
-      </c>
-      <c r="I11" s="13" t="s">
-        <v>169</v>
+      <c r="A9" s="31" t="s">
+        <v>101</v>
+      </c>
+      <c r="B9" s="32" t="s">
+        <v>286</v>
+      </c>
+      <c r="C9" s="32" t="s">
+        <v>287</v>
+      </c>
+      <c r="D9" s="32" t="s">
+        <v>288</v>
+      </c>
+      <c r="E9" s="32" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="31" t="s">
+        <v>290</v>
+      </c>
+      <c r="B10" s="32" t="s">
+        <v>291</v>
+      </c>
+      <c r="C10" s="32" t="s">
+        <v>292</v>
+      </c>
+      <c r="D10" s="32" t="s">
+        <v>293</v>
+      </c>
+      <c r="E10" s="32" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="31" t="s">
+        <v>295</v>
+      </c>
+      <c r="B11" s="32" t="s">
+        <v>296</v>
+      </c>
+      <c r="C11" s="32" t="s">
+        <v>297</v>
+      </c>
+      <c r="D11" s="32" t="s">
+        <v>298</v>
+      </c>
+      <c r="E11" s="32" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="31" t="s">
+        <v>300</v>
+      </c>
+      <c r="B12" s="32" t="s">
+        <v>301</v>
+      </c>
+      <c r="C12" s="32" t="s">
+        <v>302</v>
+      </c>
+      <c r="D12" s="32" t="s">
+        <v>303</v>
+      </c>
+      <c r="E12" s="32" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>305</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B4:B400" type="list">
-      <formula1>"Not Started,In Progress,Blocked,Completed,Cancelled"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C4:C400" type="list">
-      <formula1>"Urgent,High,Normal,Low"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>